<commit_message>
Committed changes(all TCs pased)
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataSample.xlsx
+++ b/src/test/resources/TestDataSample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\eclipse-workspace\GroceryApplication\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58619157-1FE4-4448-9CDC-503792B10CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78257D82-C2FA-4888-9239-E56DF4CC7BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{137A6599-B637-415A-9355-87A4D83D040B}"/>
   </bookViews>
@@ -59,16 +59,16 @@
     <t>adminpassword</t>
   </si>
   <si>
-    <t>tom123</t>
-  </si>
-  <si>
     <t>category</t>
   </si>
   <si>
-    <t>tomjerry233</t>
-  </si>
-  <si>
-    <t>fruits12345</t>
+    <t>fruits123456</t>
+  </si>
+  <si>
+    <t>tomjerry2334</t>
+  </si>
+  <si>
+    <t>tom1235</t>
   </si>
 </sst>
 </file>
@@ -465,7 +465,7 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -482,10 +482,10 @@
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Comitted contact and footer
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataSample.xlsx
+++ b/src/test/resources/TestDataSample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\eclipse-workspace\GroceryApplication\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78257D82-C2FA-4888-9239-E56DF4CC7BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15CD449-2E27-4B71-BCA9-2C53EEC83136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{137A6599-B637-415A-9355-87A4D83D040B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>username</t>
   </si>
@@ -62,23 +62,61 @@
     <t>category</t>
   </si>
   <si>
-    <t>fruits123456</t>
-  </si>
-  <si>
-    <t>tomjerry2334</t>
-  </si>
-  <si>
-    <t>tom1235</t>
+    <t>textareaaddress</t>
+  </si>
+  <si>
+    <t>emailaddress</t>
+  </si>
+  <si>
+    <t>phonenumber</t>
+  </si>
+  <si>
+    <t>hema villa</t>
+  </si>
+  <si>
+    <t>hema@123</t>
+  </si>
+  <si>
+    <t>deliverytime</t>
+  </si>
+  <si>
+    <t>deliverycharge</t>
+  </si>
+  <si>
+    <t>2323232323</t>
+  </si>
+  <si>
+    <t>10:00:00</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>tomjerrytom</t>
+  </si>
+  <si>
+    <t>tom1tom</t>
+  </si>
+  <si>
+    <t>fruits9876</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -101,13 +139,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -440,15 +483,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB5BB93-91E6-437C-B9A6-0C3A095F41B0}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="18.44140625" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+    <col min="9" max="9" width="12.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -467,8 +514,23 @@
       <c r="F1" t="s">
         <v>7</v>
       </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -479,16 +541,34 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{23729702-9835-4336-B882-0E860AC6A619}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>